<commit_message>
chore: add survey response
</commit_message>
<xml_diff>
--- a/igrow_survey_responses.xlsx
+++ b/igrow_survey_responses.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,6 +464,16 @@
           <t>Any suggestions or feedback for us?</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Your Name</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Community / Person who invited you</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -483,6 +493,41 @@
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-03-08 04:48:10</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>﻿One God, Three Persons</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>si jovs kasi nakatayo sya saka yung is this how you want to praise the Lord</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>doms</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>mama mo</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>